<commit_message>
feat(prompts): update VAERS prompt guidance and Supplementary File 3 to exact 11-category schema
</commit_message>
<xml_diff>
--- a/publication/manuscripts/Supplementary_File_3_VAERS_Annotation_Guidance.xlsx
+++ b/publication/manuscripts/Supplementary_File_3_VAERS_Annotation_Guidance.xlsx
@@ -8,7 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover_Sheet" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VAERS_13_Category_Schema" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VAERS_11_Category_Schema" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="General_Annotation_Rules" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
@@ -662,7 +662,7 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>13 Primary Clinical and Contextual Concept Categories (Exact Verbatim Prompt Schema)</t>
+          <t>11 Primary Clinical Feature Categories (Exact Verbatim Prompt Schema)</t>
         </is>
       </c>
       <c r="D9" s="5" t="n"/>
@@ -678,7 +678,7 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>&lt;SYM&gt;, &lt;SDX&gt;, &lt;PDX&gt;, &lt;DX&gt;, &lt;VAX&gt;, &lt;MHX&gt;, &lt;FHX&gt;, &lt;LAB&gt;, &lt;DOSE&gt;, &lt;STATUS&gt;, &lt;TX&gt;, &lt;AGE&gt;, &lt;SEX&gt;</t>
+          <t>&lt;PDX&gt;, &lt;SDX&gt;, &lt;RO&gt;, &lt;SYM&gt;, &lt;COD&gt;, &lt;LAB&gt;, &lt;STATUS&gt;, &lt;FHX&gt;, &lt;MHX&gt;, &lt;TX&gt;, &lt;VAX&gt;</t>
         </is>
       </c>
       <c r="D10" s="5" t="n"/>
@@ -694,7 +694,7 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>sym, sdx, pdx, dx, vax, mhx, fhx, lab, dose, status, tx, age, sex</t>
+          <t>pdx, sdx, ro, sym, cod, lab, status, fhx, mhx, tx, vax</t>
         </is>
       </c>
       <c r="D11" s="5" t="n"/>
@@ -758,7 +758,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:G17"/>
+  <dimension ref="B2:G15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -773,7 +773,7 @@
     <row r="2" ht="30" customHeight="1">
       <c r="B2" s="6" t="inlineStr">
         <is>
-          <t>VAERS 13 Clinical Concept Category Annotation Schema (Verbatim LLM Prompt)</t>
+          <t>VAERS 11 Clinical Feature Category Annotation Schema (Verbatim LLM Prompt)</t>
         </is>
       </c>
     </row>
@@ -812,32 +812,32 @@
     <row r="5" ht="65" customHeight="1">
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t>SYM</t>
+          <t>pDx</t>
         </is>
       </c>
       <c r="C5" s="10" t="inlineStr">
         <is>
-          <t>Symptom / Adverse-Event Sign</t>
+          <t>Primary Diagnosis</t>
         </is>
       </c>
       <c r="D5" s="11" t="inlineStr">
         <is>
-          <t>&lt;SYM&gt;</t>
+          <t>&lt;PDX&gt;</t>
         </is>
       </c>
       <c r="E5" s="12" t="inlineStr">
         <is>
-          <t>A patient-reported symptom, sign, complaint, or other clinical manifestation occurring as part of the post-vaccination adverse-event narrative.</t>
+          <t>Medical terms representing formal diagnoses or established diagnostic clinical concepts identified in the post-vaccination evaluation.</t>
         </is>
       </c>
       <c r="F5" s="12" t="inlineStr">
         <is>
-          <t>Annotate the symptom/sign itself when it is described as experienced, observed, reported, or developed in the adverse-event context and is not presented as a formal diagnosis. Prefer SYM for manifestations such as pain, fever, dizziness, rash, weakness, swelling, nausea, or other signs/symptoms when no diagnostic label is being assigned.</t>
+          <t>Annotate a medical condition as **pDx** when it appears next to trigger words indicating a formal diagnosis. Under the hierarchy rule, if a feature is first tagged as pDx, subsequent mentions keep the pDx tag even without trigger words.</t>
         </is>
       </c>
       <c r="G5" s="12" t="inlineStr">
         <is>
-          <t>symptom, symptoms, complained of, reported, experienced, developed, presented with, pain, fever, dizziness, rash, swelling, weakness, nausea, vomiting, headache, fatigue</t>
+          <t>diagnosed with, diagnosis of, diagnosed, DX, final diagnosis, determined to have, impression was</t>
         </is>
       </c>
     </row>
@@ -849,7 +849,7 @@
       </c>
       <c r="C6" s="14" t="inlineStr">
         <is>
-          <t>Confirmed AE Diagnosis</t>
+          <t>Secondary Diagnosis (Second Level)</t>
         </is>
       </c>
       <c r="D6" s="15" t="inlineStr">
@@ -859,369 +859,305 @@
       </c>
       <c r="E6" s="16" t="inlineStr">
         <is>
-          <t>A formal diagnosis or diagnosed clinical condition explicitly identified as an adverse event in the vaccination-related episode.</t>
+          <t>Medical terms describing adverse-event conditions that developed, were experienced, or were stated/suggested during the clinical episode.</t>
         </is>
       </c>
       <c r="F6" s="16" t="inlineStr">
         <is>
-          <t>Annotate a diagnosed condition as **sDx** when the narrative presents it as a confirmed/established diagnosis belonging to the adverse-event episode. Use sDx rather than SYM when the text names a diagnosis rather than a symptom, and rather than DX when the diagnosis itself is part of the adverse-event outcome being reported.</t>
+          <t>Annotate a condition as **sDx** when it appears next to trigger words indicating development, occurrence, or suggestion. Trigger words for sDx override the narrative use of the word "symptoms".</t>
         </is>
       </c>
       <c r="G6" s="16" t="inlineStr">
         <is>
-          <t>diagnosed with, diagnosis of, confirmed, final diagnosis, determined to have, diagnosed as, assessment was, impression was</t>
+          <t>develop, developed, developing, experience, experienced, state, stated, suggest, suggested, presented with</t>
         </is>
       </c>
     </row>
     <row r="7" ht="65" customHeight="1">
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>pDx</t>
+          <t>RO</t>
         </is>
       </c>
       <c r="C7" s="10" t="inlineStr">
         <is>
-          <t>Provisional AE Diagnosis</t>
+          <t>Rule-out Diagnosis</t>
         </is>
       </c>
       <c r="D7" s="11" t="inlineStr">
         <is>
-          <t>&lt;PDX&gt;</t>
+          <t>&lt;RO&gt;</t>
         </is>
       </c>
       <c r="E7" s="12" t="inlineStr">
         <is>
-          <t>A tentative, suspected, possible, or provisional diagnosis considered during evaluation of the adverse-event episode but not established as final.</t>
+          <t>Medical conditions or diagnoses considered during evaluation but explicitly ruled out, excluded, or unsupported.</t>
         </is>
       </c>
       <c r="F7" s="12" t="inlineStr">
         <is>
-          <t>Annotate a condition as **pDx** when the narrative explicitly frames it as suspected, possible, probable, provisional, differential, or otherwise uncertain during the adverse-event evaluation. Do not use pDx merely because the annotator is uncertain; uncertainty must be present in the narrative.</t>
+          <t>Annotate the condition or diagnosis that is explicitly ruled out or excluded. Do not annotate normal findings as RO unless an explicit rule-out statement is made.</t>
         </is>
       </c>
       <c r="G7" s="12" t="inlineStr">
         <is>
-          <t>possible, probable, suspected, concern for, concerning for, provisional, differential diagnosis, may have, might have, could represent, likely, presumed</t>
+          <t>r/o, ruled out, rule out, no evidence of, was considered but excluded, excluded</t>
         </is>
       </c>
     </row>
     <row r="8" ht="65" customHeight="1">
       <c r="B8" s="13" t="inlineStr">
         <is>
-          <t>DX</t>
+          <t>SYM</t>
         </is>
       </c>
       <c r="C8" s="14" t="inlineStr">
         <is>
-          <t>Diagnosis (Non-AE Context)</t>
+          <t>Symptom / Adverse-Event Sign</t>
         </is>
       </c>
       <c r="D8" s="15" t="inlineStr">
         <is>
-          <t>&lt;DX&gt;</t>
+          <t>&lt;SYM&gt;</t>
         </is>
       </c>
       <c r="E8" s="16" t="inlineStr">
         <is>
-          <t>A diagnosis or clinical condition mentioned in a diagnostic or clinical context that is not functioning as the reported adverse event, provisional AE diagnosis, medical history, or family history.</t>
+          <t>Any patient-reported symptom, sign, or adverse event manifestation that does not fall under diagnosis (pDx/sDx), rule-out, or medical history.</t>
         </is>
       </c>
       <c r="F8" s="16" t="inlineStr">
         <is>
-          <t>Annotate a diagnosis as **DX** when it is a current or contextual diagnosis but the narrative does not present it as the adverse event itself. Do not use DX for pre-existing conditions (MHx), family history (FHx), confirmed AEs (sDx), provisional AEs (pDx), symptoms (SYM), or diagnostic procedures.</t>
+          <t>Annotate the symptom/sign itself when it describes clinical manifestations (e.g., pain, fever, dizziness, rash, unresponsiveness, swelling). The resolution of specific symptoms is tagged SYM, while general outcome phrases belong to STATUS.</t>
         </is>
       </c>
       <c r="G8" s="16" t="inlineStr">
         <is>
-          <t>diagnosis, diagnosed, condition, disease, disorder, assessment, impression, clinical diagnosis</t>
+          <t>symptom, symptoms, complained of, reported, felt, sudden drop, rash, fever, dizziness, headache, nausea, pain, swelling, weakness</t>
         </is>
       </c>
     </row>
     <row r="9" ht="65" customHeight="1">
       <c r="B9" s="9" t="inlineStr">
         <is>
-          <t>VAX</t>
+          <t>CoD</t>
         </is>
       </c>
       <c r="C9" s="10" t="inlineStr">
         <is>
-          <t>Vaccine</t>
+          <t>Cause of Death</t>
         </is>
       </c>
       <c r="D9" s="11" t="inlineStr">
         <is>
-          <t>&lt;VAX&gt;</t>
+          <t>&lt;COD&gt;</t>
         </is>
       </c>
       <c r="E9" s="12" t="inlineStr">
         <is>
-          <t>A vaccine product, vaccination, immunization, or vaccine dose described as the administered or potentially causative exposure in the VAERS narrative.</t>
+          <t>A specific medical disease, condition, or event explicitly identified as causing or directly contributing to the patient's death.</t>
         </is>
       </c>
       <c r="F9" s="12" t="inlineStr">
         <is>
-          <t>Annotate the vaccine product/name or explicit vaccine reference when it identifies the immunization associated with the report. Annotate the vaccine entity itself, not surrounding administration verbs or temporal phrases.</t>
+          <t>Annotate the stated cause of death condition (e.g., "myocardial infarction"). Do not tag the word "death" alone as CoD; general death statements are tagged STATUS.</t>
         </is>
       </c>
       <c r="G9" s="12" t="inlineStr">
         <is>
-          <t>vaccine, vaccination, immunization, immunized, COVID-19 vaccine, influenza vaccine, flu vaccine, Pfizer, Moderna, Janssen, dose of vaccine, shot</t>
+          <t>cause of death, COD, died of, died from, death due to, fatal event</t>
         </is>
       </c>
     </row>
     <row r="10" ht="65" customHeight="1">
       <c r="B10" s="13" t="inlineStr">
         <is>
-          <t>MHx</t>
+          <t>Lab</t>
         </is>
       </c>
       <c r="C10" s="14" t="inlineStr">
         <is>
-          <t>Medical History</t>
+          <t>Laboratory Finding</t>
         </is>
       </c>
       <c r="D10" s="15" t="inlineStr">
         <is>
-          <t>&lt;MHX&gt;</t>
+          <t>&lt;LAB&gt;</t>
         </is>
       </c>
       <c r="E10" s="16" t="inlineStr">
         <is>
-          <t>A symptom, diagnosis, condition, or medical finding that pre-existed the vaccination/adverse-event episode or is explicitly described as part of the patient's past or chronic medical history.</t>
+          <t>Phrases describing the name of or denoting the qualitative/directional results of a laboratory, diagnostic instrument, or general test.</t>
         </is>
       </c>
       <c r="F10" s="16" t="inlineStr">
         <is>
-          <t>Annotate the historical/pre-existing clinical condition itself. Do not include contextual phrases such as "history of" when the underlying condition can be separately captured.</t>
+          <t>Annotate the test name and directional result modifier (e.g., "elevated creatine phosphokinase", "blood work"). Specific numeric values (e.g., "WBC: 114") are excluded from annotation. Diagnostic instruments (e.g., "campimetry", "CT scan") are tagged as Lab.</t>
         </is>
       </c>
       <c r="G10" s="16" t="inlineStr">
         <is>
-          <t>past medical history, medical history, PMH, history of, baseline, chronic, pre-existing, underlying condition, known condition, longstanding, prior diagnosis</t>
+          <t>laboratory, lab, blood work, physical exam, level, elevated, decreased, positive, negative, normal, abnormal, campimetry, CT, MRI, EKG</t>
         </is>
       </c>
     </row>
     <row r="11" ht="65" customHeight="1">
       <c r="B11" s="9" t="inlineStr">
         <is>
-          <t>FHx</t>
+          <t>STATUS</t>
         </is>
       </c>
       <c r="C11" s="10" t="inlineStr">
         <is>
-          <t>Family History</t>
+          <t>Patient Status / Outcome</t>
         </is>
       </c>
       <c r="D11" s="11" t="inlineStr">
         <is>
-          <t>&lt;FHX&gt;</t>
+          <t>&lt;STATUS&gt;</t>
         </is>
       </c>
       <c r="E11" s="12" t="inlineStr">
         <is>
-          <t>A disease, condition, or clinically relevant finding explicitly attributed to the patient's family members or family medical history.</t>
+          <t>Phrases describing a patient's overall clinical condition, hospital admission, discharge, recovery, deterioration, or death statement.</t>
         </is>
       </c>
       <c r="F11" s="12" t="inlineStr">
         <is>
-          <t>Annotate the condition/finding attributed to family history. Do not classify the patient's own condition as FHx.</t>
+          <t>Annotate statements describing clinical course, outcome, or hospitalization (e.g., "admitted to pediatric ER", "symptoms resolved", "recovered without sequelae", "condition deteriorated", "death").</t>
         </is>
       </c>
       <c r="G11" s="12" t="inlineStr">
         <is>
-          <t>family history, FHx, mother had, father had, sibling had, familial, hereditary, inherited, genetic predisposition</t>
+          <t>recovered, recovering, resolved, improved, worsened, deteriorated, stable, hospitalized, admitted, discharged, ER, outcome, death, died</t>
         </is>
       </c>
     </row>
     <row r="12" ht="65" customHeight="1">
       <c r="B12" s="13" t="inlineStr">
         <is>
-          <t>Lab</t>
+          <t>FHx</t>
         </is>
       </c>
       <c r="C12" s="14" t="inlineStr">
         <is>
-          <t>Laboratory Finding / Vital Sign</t>
+          <t>Family History</t>
         </is>
       </c>
       <c r="D12" s="15" t="inlineStr">
         <is>
-          <t>&lt;LAB&gt;</t>
+          <t>&lt;FHX&gt;</t>
         </is>
       </c>
       <c r="E12" s="16" t="inlineStr">
         <is>
-          <t>A laboratory test, laboratory result, vital sign, physiologic measurement, or other objective measured clinical finding.</t>
+          <t>Medical terms, conditions, or clinically relevant findings explicitly attributed to the patient's family members or family medical history.</t>
         </is>
       </c>
       <c r="F12" s="16" t="inlineStr">
         <is>
-          <t>Annotate the test/measurement and its reported result when expressed as one clinically meaningful span when practical. Include normal, abnormal, positive, negative, quantitative, and qualitative findings. Include vital signs and objective measurements when they are reported as clinical findings.</t>
+          <t>Annotate medical conditions associated with family members, including the specific family member designation when provided (e.g., "hypertension father", "coronary artery disease mother").</t>
         </is>
       </c>
       <c r="G12" s="16" t="inlineStr">
         <is>
-          <t>laboratory, lab, level, result, value, positive, negative, elevated, decreased, normal, abnormal, CBC, WBC, hemoglobin, platelet, creatinine, glucose, temperature, blood pressure, heart rate, oxygen saturation</t>
+          <t>family history, FHx, father had, mother had, sister, brother, familial, maternal, paternal</t>
         </is>
       </c>
     </row>
     <row r="13" ht="65" customHeight="1">
       <c r="B13" s="9" t="inlineStr">
         <is>
-          <t>DOSE</t>
+          <t>MHx</t>
         </is>
       </c>
       <c r="C13" s="10" t="inlineStr">
         <is>
-          <t>Dose / Lot Information</t>
+          <t>Medical History</t>
         </is>
       </c>
       <c r="D13" s="11" t="inlineStr">
         <is>
-          <t>&lt;DOSE&gt;</t>
+          <t>&lt;MHX&gt;</t>
         </is>
       </c>
       <c r="E13" s="12" t="inlineStr">
         <is>
-          <t>Vaccine dose information, dose number, amount, sequence, administration-dose descriptor, or vaccine lot/batch number.</t>
+          <t>Symptoms, conditions, diagnoses, or medical findings that pre-existed the vaccination episode or are explicitly described as past/chronic medical history.</t>
         </is>
       </c>
       <c r="F13" s="12" t="inlineStr">
         <is>
-          <t>Annotate explicit vaccine dose or lot information, including ordinal dose number and lot/batch identifier. Keep vaccine product name under VAX rather than DOSE.</t>
+          <t>Annotate historical/pre-existing conditions (e.g., "asthma", "depression", "high blood pressure"). Also annotate explicit statements reporting the absence of medical history (e.g., "no medical history").</t>
         </is>
       </c>
       <c r="G13" s="12" t="inlineStr">
         <is>
-          <t>first dose, second dose, third dose, booster, dose 1, dose 2, dose, dosage, lot, lot number, batch, batch number, 0.5 mL</t>
+          <t>past medical history, medical history, PMH, history of, baseline, chronic, pre-existing, longstanding, prior diagnosis, no medical history</t>
         </is>
       </c>
     </row>
     <row r="14" ht="65" customHeight="1">
       <c r="B14" s="13" t="inlineStr">
         <is>
-          <t>STATUS</t>
+          <t>TX</t>
         </is>
       </c>
       <c r="C14" s="14" t="inlineStr">
         <is>
-          <t>Patient Status / Outcome</t>
+          <t>Drug Product / Treatment</t>
         </is>
       </c>
       <c r="D14" s="15" t="inlineStr">
         <is>
-          <t>&lt;STATUS&gt;</t>
+          <t>&lt;TX&gt;</t>
         </is>
       </c>
       <c r="E14" s="16" t="inlineStr">
         <is>
-          <t>A statement describing the patient's clinical course, disposition, recovery, persistence, worsening, hospitalization status, disability, death status, or other outcome.</t>
+          <t>Any non-vaccine drug name, therapeutic substance class, or medication acronym appearing in the narrative.</t>
         </is>
       </c>
       <c r="F14" s="16" t="inlineStr">
         <is>
-          <t>Annotate the status/outcome expression itself. STATUS describes what happened to the patient or event over time, not the underlying symptom/diagnosis.</t>
+          <t>Annotate any drug name or class (e.g., "atenolol", "ibuprofen", "steroid shot", "penicillin"). If both brand and generic names appear, annotate each separately. If a drug appears in an allergy phrase (e.g., SYM: "allergy to penicillin"), tag the drug name additionally as TX. Also annotate explicit statements of absence ("no other concomitant medications"). Exclude dose, manufacturer, and route.</t>
         </is>
       </c>
       <c r="G14" s="16" t="inlineStr">
         <is>
-          <t>recovered, recovering, resolved, improved, worsened, stable, persistent, ongoing, hospitalized, admitted, discharged, emergency room, disability, life-threatening, outcome, died, death</t>
+          <t>treated with, treatment, therapy, given, administered, prescribed, atenolol, ibuprofen, prednisone, acetaminophen, penicillin, antibiotic, medication</t>
         </is>
       </c>
     </row>
     <row r="15" ht="65" customHeight="1">
       <c r="B15" s="9" t="inlineStr">
         <is>
-          <t>TX</t>
+          <t>VAX</t>
         </is>
       </c>
       <c r="C15" s="10" t="inlineStr">
         <is>
-          <t>Treatment / Provider / Intervention</t>
+          <t>Vaccine Product</t>
         </is>
       </c>
       <c r="D15" s="11" t="inlineStr">
         <is>
-          <t>&lt;TX&gt;</t>
+          <t>&lt;VAX&gt;</t>
         </is>
       </c>
       <c r="E15" s="12" t="inlineStr">
         <is>
-          <t>A treatment, therapeutic intervention, clinical management action, procedure used for treatment, or explicitly mentioned treating/provider service associated with management of the patient.</t>
+          <t>Any vaccine product name, immunization, or vaccine strain associated with the report.</t>
         </is>
       </c>
       <c r="F15" s="12" t="inlineStr">
         <is>
-          <t>Annotate the treatment/intervention/provider entity or therapeutic action used to manage the patient or adverse event. Do not annotate the indication as TX. Drug names used as treatment may be included as TX when explicitly administered therapeutically.</t>
+          <t>Annotate the vaccine name or specific strain (e.g., "PREVENAR 13", "INFLUVAC", "ACAM2000", "anthrax vaccine", "COVID-19 vaccine"). Include modifiers such as "vaccine", "live", or "recombinant". If a vaccine appears in an allergy phrase, tag it additionally as VAX. Exclude manufacturer, lot/batch numbers, dose number, and administration site.</t>
         </is>
       </c>
       <c r="G15" s="12" t="inlineStr">
         <is>
-          <t>treated with, treatment, therapy, given, administered, prescribed, managed with, IV fluids, acetaminophen, antihistamine, steroids, epinephrine, surgery, physician, provider, emergency department</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="65" customHeight="1">
-      <c r="B16" s="13" t="inlineStr">
-        <is>
-          <t>AGE</t>
-        </is>
-      </c>
-      <c r="C16" s="14" t="inlineStr">
-        <is>
-          <t>Patient Age</t>
-        </is>
-      </c>
-      <c r="D16" s="15" t="inlineStr">
-        <is>
-          <t>&lt;AGE&gt;</t>
-        </is>
-      </c>
-      <c r="E16" s="16" t="inlineStr">
-        <is>
-          <t>The patient's exact or approximate age or age category during the reported vaccination/adverse-event episode.</t>
-        </is>
-      </c>
-      <c r="F16" s="16" t="inlineStr">
-        <is>
-          <t>Annotate explicit references to the patient's age or age category only when they clearly refer to the patient.</t>
-        </is>
-      </c>
-      <c r="G16" s="16" t="inlineStr">
-        <is>
-          <t>year-old, years old, aged, age, infant, child, adolescent, adult, elderly, older adult</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="65" customHeight="1">
-      <c r="B17" s="9" t="inlineStr">
-        <is>
-          <t>SEX</t>
-        </is>
-      </c>
-      <c r="C17" s="10" t="inlineStr">
-        <is>
-          <t>Patient Sex</t>
-        </is>
-      </c>
-      <c r="D17" s="11" t="inlineStr">
-        <is>
-          <t>&lt;SEX&gt;</t>
-        </is>
-      </c>
-      <c r="E17" s="12" t="inlineStr">
-        <is>
-          <t>The biological sex of the patient as explicitly described in the VAERS narrative.</t>
-        </is>
-      </c>
-      <c r="F17" s="12" t="inlineStr">
-        <is>
-          <t>Annotate explicit references to the patient's biological sex only when they clearly refer to the patient.</t>
-        </is>
-      </c>
-      <c r="G17" s="12" t="inlineStr">
-        <is>
-          <t>male, female, man, woman, boy, girl</t>
+          <t>vaccine, vaccination, immunization, COVID-19 vaccine, influenza vaccine, flu vaccine, PREVENAR, INFLUVAC, ACAM2000, Pfizer, Moderna, shot</t>
         </is>
       </c>
     </row>
@@ -1239,7 +1175,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:D21"/>
+  <dimension ref="B2:D17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -1271,12 +1207,14 @@
     <row r="5" ht="50" customHeight="1">
       <c r="B5" s="18" t="inlineStr">
         <is>
-          <t>1. Use narrative context, not keyword matching.</t>
+          <t>1. Tag Hierarchy Precedence:</t>
         </is>
       </c>
       <c r="C5" s="19" t="inlineStr">
         <is>
-          <t>Trigger words and phrases are contextual clues only. A trigger word does not automatically determine an annotation.</t>
+          <t>When assigning tags, adhere to the strict hierarchy:
+MHx / FHx &gt; CoD &gt; RO &gt; pDx &gt; sDx &gt; SYM
+A higher-level classification always supersedes a lower-level one.</t>
         </is>
       </c>
       <c r="D5" s="5" t="n"/>
@@ -1284,14 +1222,12 @@
     <row r="6" ht="50" customHeight="1">
       <c r="B6" s="20" t="inlineStr">
         <is>
-          <t>2. Annotate the clinical entity, not the contextual trigger phrase.</t>
+          <t>2. Directionality &amp; Tag Persistence:</t>
         </is>
       </c>
       <c r="C6" s="21" t="inlineStr">
         <is>
-          <t>Examples:
-- "history of asthma" -&gt; annotate "asthma" as MHx.
-- "treated with acetaminophen" -&gt; annotate "acetaminophen" as TX.</t>
+          <t>Keep tag types moving forward, but not backward, in text. If a feature is first tagged as pDx, subsequent mentions retain the pDx tag even without trigger words. If first tagged as SYM and later promoted to pDx by a trigger word, the subsequent mention is tagged pDx while the earlier mention remains SYM.</t>
         </is>
       </c>
       <c r="D6" s="5" t="n"/>
@@ -1299,12 +1235,12 @@
     <row r="7" ht="50" customHeight="1">
       <c r="B7" s="18" t="inlineStr">
         <is>
-          <t>3. Use exact text spans.</t>
+          <t>3. Punctuation Rules:</t>
         </is>
       </c>
       <c r="C7" s="19" t="inlineStr">
         <is>
-          <t>Every annotated span must occur verbatim in the source narrative. Do not normalize spelling, capitalization, abbreviations, numbers, or units.</t>
+          <t>Do not include trailing periods, quotation marks, or surrounding parentheses in entity tags. Hyphens that form integral parts of noun phrases (e.g., "poison-ivy", "QT-interval") must be retained.</t>
         </is>
       </c>
       <c r="D7" s="5" t="n"/>
@@ -1312,12 +1248,12 @@
     <row r="8" ht="50" customHeight="1">
       <c r="B8" s="20" t="inlineStr">
         <is>
-          <t>4. Prefer the smallest complete clinically meaningful span.</t>
+          <t>4. Articles and Pronouns:</t>
         </is>
       </c>
       <c r="C8" s="21" t="inlineStr">
         <is>
-          <t>Do not include unnecessary surrounding words, punctuation, conjunctions, or trigger phrases.</t>
+          <t>Omit noun markers ("a", "an", "the") and personal pronouns ("he", "she", "him", "her", "the patient") from entity spans.</t>
         </is>
       </c>
       <c r="D8" s="5" t="n"/>
@@ -1325,12 +1261,12 @@
     <row r="9" ht="50" customHeight="1">
       <c r="B9" s="18" t="inlineStr">
         <is>
-          <t>5. Do not infer unsupported clinical relationships.</t>
+          <t>5. Auxiliary Verbs:</t>
         </is>
       </c>
       <c r="C9" s="19" t="inlineStr">
         <is>
-          <t>Use only information expressed or clearly established in the narrative. Do not infer causality, chronology, diagnosis certainty, medical history, or treatment role solely from medical knowledge.</t>
+          <t>Exclude auxiliary verbs ("can", "could", "will", "would", "had", "was", "were", "been") unless essential for clarity in negated spans (e.g., in "did not experience anaphylaxis", include "did").</t>
         </is>
       </c>
       <c r="D9" s="5" t="n"/>
@@ -1338,12 +1274,12 @@
     <row r="10" ht="50" customHeight="1">
       <c r="B10" s="20" t="inlineStr">
         <is>
-          <t>6. Do not annotate the same text span with multiple categories.</t>
+          <t>6. Hypothetical and Conditional Statements:</t>
         </is>
       </c>
       <c r="C10" s="21" t="inlineStr">
         <is>
-          <t>Choose the category that best represents the role of that occurrence in its local narrative context.</t>
+          <t>Do not annotate hypothetical, conditional, or precautionary phrases (e.g., do not annotate "if heart palpitations worsen return to ER").</t>
         </is>
       </c>
       <c r="D10" s="5" t="n"/>
@@ -1351,25 +1287,26 @@
     <row r="11" ht="50" customHeight="1">
       <c r="B11" s="18" t="inlineStr">
         <is>
-          <t>7. Do not create overlapping or nested annotations.</t>
-        </is>
-      </c>
-      <c r="C11" s="19" t="inlineStr"/>
+          <t>7. Parenthetical Text:</t>
+        </is>
+      </c>
+      <c r="C11" s="19" t="inlineStr">
+        <is>
+          <t>- If parenthetical text contains relevant clinical concepts or acronyms (e.g., "computed tomography (CAT) scan", "Good Syndrome (GS)"), tag each entity separately without parentheses.
+- If parenthetical text contains irrelevant metadata (e.g., manufacturer name, batch numbers), do not annotate it.</t>
+        </is>
+      </c>
       <c r="D11" s="5" t="n"/>
     </row>
     <row r="12" ht="50" customHeight="1">
       <c r="B12" s="20" t="inlineStr">
         <is>
-          <t>8. SYM vs sDx vs pDx vs DX must follow the narrative role.</t>
+          <t>8. Inclusive Clinical Concept Spans:</t>
         </is>
       </c>
       <c r="C12" s="21" t="inlineStr">
         <is>
-          <t>- SYM = symptom/sign/complaint without a formal diagnostic role.
-- sDx = established/confirmed diagnosis functioning as an adverse event in the reported episode.
-- pDx = tentative/suspected/provisional diagnosis in the adverse-event episode.
-- DX = diagnosis in a current/contextual non-AE role.
-Do not convert a symptom into a diagnosis based only on medical knowledge.</t>
+          <t>Include all essential clinical adjectives, anatomical modifiers, negations, and syntactic modifiers within a single entity span (e.g., "coronary heart disease", "severe asthma", "no nausea", "inflammatory myopathy without inclusive bodies").</t>
         </is>
       </c>
       <c r="D12" s="5" t="n"/>
@@ -1377,12 +1314,16 @@
     <row r="13" ht="50" customHeight="1">
       <c r="B13" s="18" t="inlineStr">
         <is>
-          <t>9. sDx vs pDx is determined by diagnostic certainty expressed in the text.</t>
+          <t>9. Clinical Modifiers:</t>
         </is>
       </c>
       <c r="C13" s="19" t="inlineStr">
         <is>
-          <t>A diagnosis is pDx only when the narrative itself indicates uncertainty, suspicion, possibility, probability, or provisional status.</t>
+          <t>- Include modifiers indicating onset, continuation, or conclusion ("started", "began", "continued", "resolved", "became").
+- Include subjective feeling inflections ("felt tired", "feeling sick").
+- Include clinical severity descriptors ("clinically significant", "disabling").
+- Include uncertainty modifiers ("possible anaphylaxis").
+- Exclude overly general non-clinical modifiers (e.g., "routine").</t>
         </is>
       </c>
       <c r="D13" s="5" t="n"/>
@@ -1390,14 +1331,12 @@
     <row r="14" ht="50" customHeight="1">
       <c r="B14" s="20" t="inlineStr">
         <is>
-          <t>10. MHx and FHx take precedence when history is explicit.</t>
+          <t>10. Associated Features:</t>
         </is>
       </c>
       <c r="C14" s="21" t="inlineStr">
         <is>
-          <t>- MHx = patient's own pre-existing/historical condition.
-- FHx = condition attributed to family members/family history.
-Do not relabel these occurrences as SYM, sDx, pDx, or DX solely because the same condition could be clinically relevant to the current event.</t>
+          <t>In structures such as "Medical condition with [feature 1] and [feature 2]", annotate each distinct associated feature separately with the parent condition's tag type.</t>
         </is>
       </c>
       <c r="D14" s="5" t="n"/>
@@ -1405,14 +1344,12 @@
     <row r="15" ht="50" customHeight="1">
       <c r="B15" s="18" t="inlineStr">
         <is>
-          <t>11. VAX identifies the vaccine exposure, not the timing or dose descriptor.</t>
+          <t>11. Trigger Words:</t>
         </is>
       </c>
       <c r="C15" s="19" t="inlineStr">
         <is>
-          <t>Example: "second dose of Pfizer vaccine"
-- "second dose" -&gt; DOSE
-- "Pfizer vaccine" -&gt; VAX</t>
+          <t>Trigger words (e.g., "diagnosed", "experienced", "developed") should not be included at the beginning of an annotation, but must be preserved if they occur in the middle of a concept or in explicit statements of absence (e.g., "no medical history reported").</t>
         </is>
       </c>
       <c r="D15" s="5" t="n"/>
@@ -1420,12 +1357,12 @@
     <row r="16" ht="50" customHeight="1">
       <c r="B16" s="20" t="inlineStr">
         <is>
-          <t>12. DOSE includes vaccine sequence and lot information.</t>
+          <t>12. Annotating Lists:</t>
         </is>
       </c>
       <c r="C16" s="21" t="inlineStr">
         <is>
-          <t>Dose number, amount, booster designation, and lot/batch identifiers belong to DOSE when explicitly stated.</t>
+          <t>Annotate each item in a list separately while propagating shared modifiers before or after the list (e.g., "decreased muscle tone", "pallor", "altered consciousness", "drowsiness").</t>
         </is>
       </c>
       <c r="D16" s="5" t="n"/>
@@ -1433,89 +1370,33 @@
     <row r="17" ht="50" customHeight="1">
       <c r="B17" s="18" t="inlineStr">
         <is>
-          <t>13. Lab includes objective laboratory findings and vital signs.</t>
+          <t>13. Strict 11-Category Boundary:</t>
         </is>
       </c>
       <c r="C17" s="19" t="inlineStr">
         <is>
-          <t>Diagnostic labels inferred from those findings should not be added unless explicitly stated elsewhere in the narrative.</t>
+          <t>Annotate ONLY the 11 categories defined above. Do not invent or add extraneous categories.</t>
         </is>
       </c>
       <c r="D17" s="5" t="n"/>
     </row>
-    <row r="18" ht="50" customHeight="1">
-      <c r="B18" s="20" t="inlineStr">
-        <is>
-          <t>14. STATUS describes course, disposition, or outcome.</t>
-        </is>
-      </c>
-      <c r="C18" s="21" t="inlineStr">
-        <is>
-          <t>Do not label the underlying symptom or diagnosis as STATUS merely because its course or outcome is discussed.</t>
-        </is>
-      </c>
-      <c r="D18" s="5" t="n"/>
-    </row>
-    <row r="19" ht="50" customHeight="1">
-      <c r="B19" s="18" t="inlineStr">
-        <is>
-          <t>15. TX includes therapeutic management/intervention.</t>
-        </is>
-      </c>
-      <c r="C19" s="19" t="inlineStr">
-        <is>
-          <t>Annotate what was done to treat or manage the patient. Do not label the condition being treated as TX.</t>
-        </is>
-      </c>
-      <c r="D19" s="5" t="n"/>
-    </row>
-    <row r="20" ht="50" customHeight="1">
-      <c r="B20" s="20" t="inlineStr">
-        <is>
-          <t>16. Repeated mentions may be annotated separately.</t>
-        </is>
-      </c>
-      <c r="C20" s="21" t="inlineStr">
-        <is>
-          <t>If the same concept appears multiple times, annotate each explicit occurrence according to its local context.</t>
-        </is>
-      </c>
-      <c r="D20" s="5" t="n"/>
-    </row>
-    <row r="21" ht="50" customHeight="1">
-      <c r="B21" s="18" t="inlineStr">
-        <is>
-          <t>17. Annotate only the 13 VAERS categories defined above.</t>
-        </is>
-      </c>
-      <c r="C21" s="19" t="inlineStr">
-        <is>
-          <t>Do not invent or add additional categories.</t>
-        </is>
-      </c>
-      <c r="D21" s="5" t="n"/>
-    </row>
   </sheetData>
-  <mergeCells count="19">
+  <mergeCells count="15">
+    <mergeCell ref="C12:D12"/>
     <mergeCell ref="C6:D6"/>
+    <mergeCell ref="C7:D7"/>
+    <mergeCell ref="C10:D10"/>
+    <mergeCell ref="C8:D8"/>
     <mergeCell ref="C15:D15"/>
+    <mergeCell ref="C16:D16"/>
+    <mergeCell ref="C11:D11"/>
     <mergeCell ref="C5:D5"/>
     <mergeCell ref="C14:D14"/>
+    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="C9:D9"/>
+    <mergeCell ref="C17:D17"/>
+    <mergeCell ref="B2:D2"/>
     <mergeCell ref="C4:D4"/>
-    <mergeCell ref="C20:D20"/>
-    <mergeCell ref="C10:D10"/>
-    <mergeCell ref="C16:D16"/>
-    <mergeCell ref="C9:D9"/>
-    <mergeCell ref="C12:D12"/>
-    <mergeCell ref="C21:D21"/>
-    <mergeCell ref="C11:D11"/>
-    <mergeCell ref="C17:D17"/>
-    <mergeCell ref="C8:D8"/>
-    <mergeCell ref="C7:D7"/>
-    <mergeCell ref="C19:D19"/>
-    <mergeCell ref="C13:D13"/>
-    <mergeCell ref="C18:D18"/>
-    <mergeCell ref="B2:D2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>